<commit_message>
결과 파일 업데이트 2026-08-09 08:37
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260809.xlsx
+++ b/results/andar_할인율모니터링_20260809.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>256</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>256</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>256</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6,342</t>
+          <t>6,343</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1,078</t>
+          <t>1,079</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>314</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>10,267</t>
+          <t>10,268</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>1,926</t>
+          <t>1,927</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>224</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>168</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>33</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.4</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>168</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>260</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>1,926</t>
+          <t>1,927</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>223</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>764</t>
+          <t>767</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">

</xml_diff>